<commit_message>
se realizaron modificaciones en bugs encontrados app spotify
</commit_message>
<xml_diff>
--- a/bugs/Bugs encontrados app Spotify.xlsx
+++ b/bugs/Bugs encontrados app Spotify.xlsx
@@ -1,12 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="588" yWindow="588" windowWidth="21852" windowHeight="8676"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
@@ -118,23 +121,31 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -142,7 +153,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -152,7 +163,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -166,34 +183,30 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -201,7 +214,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -391,157 +404,161 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="16.75"/>
-    <col customWidth="1" min="2" max="2" width="22.38"/>
-    <col customWidth="1" min="3" max="3" width="22.25"/>
-    <col customWidth="1" min="4" max="4" width="22.0"/>
-    <col customWidth="1" min="5" max="5" width="10.5"/>
-    <col customWidth="1" min="6" max="6" width="23.88"/>
+    <col min="1" max="1" width="19.5546875" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="23.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="27.6">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" ht="55.8" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" ht="66">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" ht="52.8">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="52.8">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="52.8">
+      <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="66">
+      <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="3"/>
+      <c r="F7" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
realice modificaciones en bugs encontrados app Spotify
</commit_message>
<xml_diff>
--- a/bugs/Bugs encontrados app Spotify.xlsx
+++ b/bugs/Bugs encontrados app Spotify.xlsx
@@ -1,12 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="588" yWindow="588" windowWidth="21852" windowHeight="8676"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
@@ -118,23 +121,31 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -142,7 +153,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -152,7 +163,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -166,34 +183,30 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -201,7 +214,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -391,157 +404,161 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="16.75"/>
-    <col customWidth="1" min="2" max="2" width="22.38"/>
-    <col customWidth="1" min="3" max="3" width="22.25"/>
-    <col customWidth="1" min="4" max="4" width="22.0"/>
-    <col customWidth="1" min="5" max="5" width="10.5"/>
-    <col customWidth="1" min="6" max="6" width="23.88"/>
+    <col min="1" max="1" width="20.5546875" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="6" max="6" width="23.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="27.6">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" ht="53.4" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" ht="57.6" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" ht="52.8" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="52.8" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="52.8" customHeight="1">
+      <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="66" customHeight="1">
+      <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="3"/>
+      <c r="F7" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>